<commit_message>
Metales SQ: policarbonato rectangular de 8 crestas y ancho 1,07 en rectangular de segunda
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/metalessq-whatsapp/textos-catalogo-whatsapp.xlsx
+++ b/metalessq-whatsapp/textos-catalogo-whatsapp.xlsx
@@ -4567,7 +4567,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>Lámina rectangular #28 aluminizada para techo. Espesor: 0,31 mm. Medidas: largo 3,66 m. Material de segunda: mismas medidas, a menor precio. Decinos la cantidad y te cotizamos. Retirás en Coronado, Tibás, Alajuela y Guápiles.</t>
+          <t>Lámina rectangular #28 aluminizada para techo. Espesor: 0,31 mm. Medidas: largo 3,66 m · ancho 1,07 m. Material de segunda: mismas medidas, a menor precio. Decinos la cantidad y te cotizamos. Retirás en Coronado, Tibás, Alajuela y Guápiles.</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
@@ -4594,7 +4594,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>Lámina rectangular #28 esmaltada para techo. Colores: verde, rojo y blanco. Espesor: 0,32 y 0,35 mm. Medidas: largo 3,66 m. Material de segunda: mismas medidas, a menor precio. Decinos la cantidad y te cotizamos. Retirás en Coronado, Tibás, Alajuela y Guápiles.</t>
+          <t>Lámina rectangular #28 esmaltada para techo. Colores: verde, rojo y blanco. Espesor: 0,32 y 0,35 mm. Medidas: largo 3,66 m · ancho 1,07 m. Material de segunda: mismas medidas, a menor precio. Decinos la cantidad y te cotizamos. Retirás en Coronado, Tibás, Alajuela y Guápiles.</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
@@ -4621,7 +4621,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>Lámina rectangular #26 esmaltada para techo. Colores: verde, rojo, blanco y naranja. Espesor: 0,40 y 0,45 mm. Medidas: largo 3,66 m. Material de segunda: mismas medidas, a menor precio. Decinos la cantidad y te cotizamos. Retirás en Coronado, Tibás, Alajuela y Guápiles.</t>
+          <t>Lámina rectangular #26 esmaltada para techo. Colores: verde, rojo, blanco y naranja. Espesor: 0,40 y 0,45 mm. Medidas: largo 3,66 m · ancho 1,07 m. Material de segunda: mismas medidas, a menor precio. Decinos la cantidad y te cotizamos. Retirás en Coronado, Tibás, Alajuela y Guápiles.</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
@@ -4648,7 +4648,7 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>Lámina rectangular #26 esmaltada corta para techo. Colores: verde, blanco y rojo. Espesor: 0,40 mm. Medidas: largo 3,60 m. Material de segunda: mismas medidas, a menor precio. Decinos la cantidad y te cotizamos. Retirás en Coronado, Tibás, Alajuela y Guápiles.</t>
+          <t>Lámina rectangular #26 esmaltada corta para techo. Colores: verde, blanco y rojo. Espesor: 0,40 mm. Medidas: largo 3,60 m · ancho 1,07 m. Material de segunda: mismas medidas, a menor precio. Decinos la cantidad y te cotizamos. Retirás en Coronado, Tibás, Alajuela y Guápiles.</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
@@ -4675,7 +4675,7 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>Lámina corta galvanizada para techo. Espesor: 0,35 y 0,40 mm. Medidas: largo 1,83 m. Material de segunda: mismas medidas, a menor precio. Decinos la cantidad y te cotizamos. Retirás en Coronado, Tibás, Alajuela y Guápiles.</t>
+          <t>Lámina corta galvanizada para techo. Espesor: 0,35 y 0,40 mm. Medidas: largo 1,83 m · ancho 1,07 m. Material de segunda: mismas medidas, a menor precio. Decinos la cantidad y te cotizamos. Retirás en Coronado, Tibás, Alajuela y Guápiles.</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">

</xml_diff>

<commit_message>
Metales SQ: ancho 1,07 en rectangular, lisa y policarbonato
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/metalessq-whatsapp/textos-catalogo-whatsapp.xlsx
+++ b/metalessq-whatsapp/textos-catalogo-whatsapp.xlsx
@@ -1381,7 +1381,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Lámina rectangular #28 aluminizada para techo. Espesor: 0,31 mm. Medidas: largo 3,66 m. Decinos la cantidad y te cotizamos. Retirás en Coronado, Tibás, Alajuela y Guápiles.</t>
+          <t>Lámina rectangular #28 aluminizada para techo. Espesor: 0,31 mm. Medidas: largo 3,66 m · ancho 1,07 m. Decinos la cantidad y te cotizamos. Retirás en Coronado, Tibás, Alajuela y Guápiles.</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -1408,7 +1408,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Lámina rectangular #28 esmaltada para techo. Colores: verde, rojo y blanco. Espesor: 0,32 y 0,35 mm. Medidas: largo 3,66 m. Decinos la cantidad y te cotizamos. Retirás en Coronado, Tibás, Alajuela y Guápiles.</t>
+          <t>Lámina rectangular #28 esmaltada para techo. Colores: verde, rojo y blanco. Espesor: 0,32 y 0,35 mm. Medidas: largo 3,66 m · ancho 1,07 m. Decinos la cantidad y te cotizamos. Retirás en Coronado, Tibás, Alajuela y Guápiles.</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -1435,7 +1435,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Lámina rectangular #26 esmaltada para techo. Colores: verde, rojo y blanco. Espesor: 0,40 y 0,45 mm. Medidas: largo 3,66 m. Decinos la cantidad y te cotizamos. Retirás en Coronado, Tibás, Alajuela y Guápiles.</t>
+          <t>Lámina rectangular #26 esmaltada para techo. Colores: verde, rojo y blanco. Espesor: 0,40 y 0,45 mm. Medidas: largo 3,66 m · ancho 1,07 m. Decinos la cantidad y te cotizamos. Retirás en Coronado, Tibás, Alajuela y Guápiles.</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -1462,7 +1462,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Lámina lisa #26 de 6 m. Lámina plana para hojalatería. Color: blanca, teja, verde, roja y galvanizada. Decinos la cantidad y te cotizamos. Retirás en Coronado, Tibás, Alajuela y Guápiles.</t>
+          <t>Lámina lisa #26 de 6 m. Lámina plana para hojalatería · ancho 1,07 m. Color: blanca, teja, verde, roja y galvanizada. Decinos la cantidad y te cotizamos. Retirás en Coronado, Tibás, Alajuela y Guápiles.</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -1489,7 +1489,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Policarbonato ondulada. 3,66 × 0,81 m. Decinos la cantidad y te cotizamos. Retirás en Coronado, Tibás, Alajuela y Guápiles.</t>
+          <t>Policarbonato ondulada. 3,66 × 1,07 m. Decinos la cantidad y te cotizamos. Retirás en Coronado, Tibás, Alajuela y Guápiles.</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -1516,7 +1516,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Policarbonato rectangular. 3,66 × 0,81 m. Decinos la cantidad y te cotizamos. Retirás en Coronado, Tibás, Alajuela y Guápiles.</t>
+          <t>Policarbonato rectangular. 3,66 × 1,07 m. Decinos la cantidad y te cotizamos. Retirás en Coronado, Tibás, Alajuela y Guápiles.</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -4702,7 +4702,7 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>Lámina lisa #26 de 6 m. Lámina plana. Color: blanca y roja. Material de segunda: mismas medidas, a menor precio. Decinos la cantidad y te cotizamos. Retirás en Coronado, Tibás, Alajuela y Guápiles.</t>
+          <t>Lámina lisa #26 de 6 m. Lámina plana · ancho 1,07 m. Color: blanca y roja. Material de segunda: mismas medidas, a menor precio. Decinos la cantidad y te cotizamos. Retirás en Coronado, Tibás, Alajuela y Guápiles.</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
@@ -4729,7 +4729,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>Policarbonato ondulada. 3,66 × 0,81 m. Material de segunda: mismas medidas, a menor precio. Decinos la cantidad y te cotizamos. Retirás en Coronado, Tibás, Alajuela y Guápiles.</t>
+          <t>Policarbonato ondulada. 3,66 × 1,07 m. Material de segunda: mismas medidas, a menor precio. Decinos la cantidad y te cotizamos. Retirás en Coronado, Tibás, Alajuela y Guápiles.</t>
         </is>
       </c>
       <c r="D160" t="inlineStr">
@@ -4756,7 +4756,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>Policarbonato rectangular. 3,66 × 0,81 m. Material de segunda: mismas medidas, a menor precio. Decinos la cantidad y te cotizamos. Retirás en Coronado, Tibás, Alajuela y Guápiles.</t>
+          <t>Policarbonato rectangular. 3,66 × 1,07 m. Material de segunda: mismas medidas, a menor precio. Decinos la cantidad y te cotizamos. Retirás en Coronado, Tibás, Alajuela y Guápiles.</t>
         </is>
       </c>
       <c r="D161" t="inlineStr">

</xml_diff>